<commit_message>
fix(appium): make the 2 previously-skipped tests actually pass
- test_appium_017 (authenticated tab bar): was only skipped because the
  Appium run defaulted to placeholder test credentials. Verified manually
  that the disposable QA account logs in fine on the native APK (the earlier
  failures were specific to the web/Selenium path) — no code change needed,
  just stopped overriding VOXIRA_TEST_EMAIL to the placeholder for Appium.
- test_appium_018 (mic permission dialog): was an unconditional skip. Now
  logs in, revokes RECORD_AUDIO first (grants persist across pm clear, so a
  prior run would otherwise make this a silent no-op), navigates to the
  Speech tab, taps Start Recording, and accepts the resulting system dialog.

Full suite: 20/20 Android Appium tests passing, 0 failed, 0 skipped.
Project-wide: 1088/1088 tests, 100.0% pass rate.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/selenium_model/ALL_TEST_CASES_FLAT_REPORT.xlsx
+++ b/selenium_model/ALL_TEST_CASES_FLAT_REPORT.xlsx
@@ -32,7 +32,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,11 +47,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -73,15 +68,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3436,11 +3428,11 @@
         </is>
       </c>
       <c r="I62" s="2" t="n">
-        <v>5.453</v>
+        <v>5.436</v>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:07:46</t>
+          <t>2026-08-03 00:35:22</t>
         </is>
       </c>
     </row>
@@ -3484,11 +3476,11 @@
         </is>
       </c>
       <c r="I63" s="2" t="n">
-        <v>6.167</v>
+        <v>6.201</v>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:08:13</t>
+          <t>2026-08-03 00:35:48</t>
         </is>
       </c>
     </row>
@@ -3532,11 +3524,11 @@
         </is>
       </c>
       <c r="I64" s="2" t="n">
-        <v>9.125999999999999</v>
+        <v>9.164999999999999</v>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:08:42</t>
+          <t>2026-08-03 00:36:19</t>
         </is>
       </c>
     </row>
@@ -3580,11 +3572,11 @@
         </is>
       </c>
       <c r="I65" s="2" t="n">
-        <v>11.271</v>
+        <v>11.358</v>
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:09:15</t>
+          <t>2026-08-03 00:36:51</t>
         </is>
       </c>
     </row>
@@ -3628,11 +3620,11 @@
         </is>
       </c>
       <c r="I66" s="2" t="n">
-        <v>9.301</v>
+        <v>8.659000000000001</v>
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:09:47</t>
+          <t>2026-08-03 00:37:21</t>
         </is>
       </c>
     </row>
@@ -3676,11 +3668,11 @@
         </is>
       </c>
       <c r="I67" s="2" t="n">
-        <v>11.398</v>
+        <v>10.803</v>
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:10:23</t>
+          <t>2026-08-03 00:37:54</t>
         </is>
       </c>
     </row>
@@ -3724,11 +3716,11 @@
         </is>
       </c>
       <c r="I68" s="2" t="n">
-        <v>12.004</v>
+        <v>12.191</v>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:10:56</t>
+          <t>2026-08-03 00:38:26</t>
         </is>
       </c>
     </row>
@@ -3772,11 +3764,11 @@
         </is>
       </c>
       <c r="I69" s="2" t="n">
-        <v>9.781000000000001</v>
+        <v>9.837</v>
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:11:31</t>
+          <t>2026-08-03 00:38:58</t>
         </is>
       </c>
     </row>
@@ -3820,11 +3812,11 @@
         </is>
       </c>
       <c r="I70" s="2" t="n">
-        <v>8.298999999999999</v>
+        <v>8.382</v>
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:12:02</t>
+          <t>2026-08-03 00:39:28</t>
         </is>
       </c>
     </row>
@@ -3868,11 +3860,11 @@
         </is>
       </c>
       <c r="I71" s="2" t="n">
-        <v>12.104</v>
+        <v>11.993</v>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:12:34</t>
+          <t>2026-08-03 00:40:01</t>
         </is>
       </c>
     </row>
@@ -3916,11 +3908,11 @@
         </is>
       </c>
       <c r="I72" s="2" t="n">
-        <v>10.159</v>
+        <v>10.003</v>
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:13:04</t>
+          <t>2026-08-03 00:40:32</t>
         </is>
       </c>
     </row>
@@ -3964,11 +3956,11 @@
         </is>
       </c>
       <c r="I73" s="2" t="n">
-        <v>10.764</v>
+        <v>11.546</v>
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:13:38</t>
+          <t>2026-08-03 00:41:04</t>
         </is>
       </c>
     </row>
@@ -4012,11 +4004,11 @@
         </is>
       </c>
       <c r="I74" s="2" t="n">
-        <v>11.257</v>
+        <v>10.947</v>
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:14:12</t>
+          <t>2026-08-03 00:41:36</t>
         </is>
       </c>
     </row>
@@ -4060,11 +4052,11 @@
         </is>
       </c>
       <c r="I75" s="2" t="n">
-        <v>8.695</v>
+        <v>8.532999999999999</v>
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:14:43</t>
+          <t>2026-08-03 00:42:05</t>
         </is>
       </c>
     </row>
@@ -4108,11 +4100,11 @@
         </is>
       </c>
       <c r="I76" s="2" t="n">
-        <v>8.617000000000001</v>
+        <v>8.66</v>
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:15:13</t>
+          <t>2026-08-03 00:42:36</t>
         </is>
       </c>
     </row>
@@ -4156,99 +4148,107 @@
         </is>
       </c>
       <c r="I77" s="2" t="n">
-        <v>13.593</v>
+        <v>12.881</v>
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:15:49</t>
+          <t>2026-08-03 00:43:10</t>
         </is>
       </c>
     </row>
     <row r="78" ht="16" customHeight="1">
-      <c r="A78" s="3" t="n">
+      <c r="A78" s="2" t="n">
         <v>77</v>
       </c>
-      <c r="B78" s="3" t="inlineStr">
+      <c r="B78" s="2" t="inlineStr">
         <is>
           <t>tests/test_appium.py::test_appium_017_tab_bar_tabs_count</t>
         </is>
       </c>
-      <c r="C78" s="3" t="inlineStr">
+      <c r="C78" s="2" t="inlineStr">
         <is>
           <t>Appium</t>
         </is>
       </c>
-      <c r="D78" s="3" t="inlineStr">
+      <c r="D78" s="2" t="inlineStr">
         <is>
           <t>Appium</t>
         </is>
       </c>
-      <c r="E78" s="3" t="inlineStr">
+      <c r="E78" s="2" t="inlineStr">
         <is>
           <t>APPIUM-017: Bottom tab bar shows 5 tabs after login (authenticated)</t>
         </is>
       </c>
-      <c r="F78" s="3" t="inlineStr">
+      <c r="F78" s="2" t="inlineStr">
         <is>
           <t>5 tab labels visible (Home, Speech, Goals, Earn, Profile)</t>
         </is>
       </c>
-      <c r="G78" s="3" t="n"/>
-      <c r="H78" s="3" t="inlineStr">
-        <is>
-          <t>Skipped</t>
-        </is>
-      </c>
-      <c r="I78" s="3" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="J78" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-03 00:16:11</t>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>visible_tabs=['Home', 'Speech', 'Goals', 'Earn', 'Profile']</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="n">
+        <v>16.769</v>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03 00:43:47</t>
         </is>
       </c>
     </row>
     <row r="79" ht="16" customHeight="1">
-      <c r="A79" s="3" t="n">
+      <c r="A79" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="B79" s="3" t="inlineStr">
+      <c r="B79" s="2" t="inlineStr">
         <is>
           <t>tests/test_appium.py::test_appium_018_mic_permission_dialog_android</t>
         </is>
       </c>
-      <c r="C79" s="3" t="inlineStr">
+      <c r="C79" s="2" t="inlineStr">
         <is>
           <t>Appium</t>
         </is>
       </c>
-      <c r="D79" s="3" t="inlineStr">
+      <c r="D79" s="2" t="inlineStr">
         <is>
           <t>Appium</t>
         </is>
       </c>
-      <c r="E79" s="3" t="inlineStr">
+      <c r="E79" s="2" t="inlineStr">
         <is>
           <t>APPIUM-018: Mic permission dialog can be accepted on Android</t>
         </is>
       </c>
-      <c r="F79" s="3" t="inlineStr">
-        <is>
-          <t>Permission dialog appears and can be accepted without crash</t>
-        </is>
-      </c>
-      <c r="G79" s="3" t="n"/>
-      <c r="H79" s="3" t="inlineStr">
-        <is>
-          <t>Skipped</t>
-        </is>
-      </c>
-      <c r="I79" s="3" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="J79" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-03 00:16:33</t>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Permission dialog appears when requesting RECORD_AUDIO and can be accepted</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>dialog_shown=True, accepted=True</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="n">
+        <v>20.46</v>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03 00:44:27</t>
         </is>
       </c>
     </row>
@@ -4292,11 +4292,11 @@
         </is>
       </c>
       <c r="I80" s="2" t="n">
-        <v>16.338</v>
+        <v>16.322</v>
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:17:09</t>
+          <t>2026-08-03 00:45:03</t>
         </is>
       </c>
     </row>
@@ -4340,11 +4340,11 @@
         </is>
       </c>
       <c r="I81" s="2" t="n">
-        <v>6.194</v>
+        <v>6.203</v>
       </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03 00:17:37</t>
+          <t>2026-08-03 00:45:29</t>
         </is>
       </c>
     </row>

</xml_diff>